<commit_message>
Soudanais et tchadien classés à leur pays
Les deux lignes se rangeaient sous « A » avec l'arabe littéraire. Elles
apparaissent maintenant à « Soudanais » et « Tchadien », là où on les
cherche à l'accueil. La mention entre parenthèses garde la recherche
« arabe » opérante sur les trois lignes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_traduction.xlsx
+++ b/data_traduction.xlsx
@@ -2498,7 +2498,6 @@
           <t>Forme écrite commune à tout le monde arabe</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>rtl</t>
@@ -2598,7 +2597,7 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>Arabe soudanais</t>
+          <t>Soudanais (Arabe soudanais)</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -2651,7 +2650,6 @@
           <t>Non traduit</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" s="23" t="inlineStr">
         <is>
           <t>هل لديك موعد مقابلة في مكتب OFPRA؟</t>
@@ -2693,7 +2691,7 @@
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>Arabe tchadien</t>
+          <t>Tchadien (Arabe tchadien)</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -2746,7 +2744,6 @@
           <t>Non traduit</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" s="23" t="inlineStr">
         <is>
           <t>هل لديك موعد مقابلة في مكتب OFPRA؟</t>

</xml_diff>

<commit_message>
Drapeaux kurde et tibétain rattachés à leurs langues
Dernière pièce manquante : les deux images étaient dans flags/ mais les
cases Drapeaux restaient vides, donc rien ne s'affichait.

Les 40 langues qui ont un drapeau pointent maintenant vers un fichier
présent dans flags/, vérifié un par un. Seul l'arabe littéraire reste
sans drapeau, faute de pays correspondant.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_traduction.xlsx
+++ b/data_traduction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eulalie.saisset\Documents\1 - Admin\8 - Perso\Oasis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{21E11140-98CF-4424-9751-3BC1AC2FA7AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{EB11B65A-6BAD-4DF3-9B39-0FEB10074DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4545" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1274,7 +1274,63 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="43">
+  <dxfs count="47">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1696,34 +1752,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
@@ -1831,34 +1859,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BBC3B8F8-078D-484B-B353-2EAA17FE9B13}" name="Table1" displayName="Table1" ref="A1:Y42" totalsRowShown="0" headerRowDxfId="41" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BBC3B8F8-078D-484B-B353-2EAA17FE9B13}" name="Table1" displayName="Table1" ref="A1:Y42" totalsRowShown="0" headerRowDxfId="45" dataDxfId="12">
   <autoFilter ref="A1:Y42" xr:uid="{BBC3B8F8-078D-484B-B353-2EAA17FE9B13}"/>
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{B71FE2A2-594B-49D5-BF3E-0B87B4A1CCB0}" name="Code" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{99066ED7-FB73-4CE5-BD6D-68B2A16797E7}" name="Langue_fr" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{C5E5BAF6-A992-496A-BC66-B4AF9AA92DD0}" name="Langue_native" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{908B39BA-3596-4F72-8BCF-3C1B2FCCCEF3}" name="Pays" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{1B72A290-5C1E-44A6-A447-200ACF6716B7}" name="Drapeaux" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{C563CC17-226F-4704-AF96-E07E25D95B6B}" name="Sens" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{0725BA7C-155A-4894-A65C-F1E296BE4C5E}" name="Statut1" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{4993FA21-15CF-4114-922A-393B03A69DCE}" name="Statut2" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{14C38812-CC74-499C-952C-386D47399C0E}" name="Statut3" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{877139FF-4465-413E-B07D-E4A10D59F0E3}" name="Statut4" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{F1D42B2E-DB2B-42AF-B635-840FD5759FE4}" name="Statut5" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{14E090AC-24BB-4F19-9BCA-D2ABE2BE0E4F}" name="Statut6" dataDxfId="18"/>
-    <tableColumn id="13" xr3:uid="{AE6452AC-3435-467C-A6C1-280E1815DBC4}" name="Contact" dataDxfId="17"/>
-    <tableColumn id="14" xr3:uid="{3083C17E-EDF2-413A-B542-7CAC44270421}" name="P1" dataDxfId="16"/>
-    <tableColumn id="15" xr3:uid="{326B870C-034B-4A48-A0E2-3B9AA7D7030D}" name="P2" dataDxfId="15"/>
-    <tableColumn id="16" xr3:uid="{25CB2B33-4D8A-449D-8554-52DEFA418EA8}" name="P3" dataDxfId="14"/>
-    <tableColumn id="17" xr3:uid="{90A3021E-E98D-443C-BB21-CF012B0830DB}" name="P4" dataDxfId="13"/>
-    <tableColumn id="18" xr3:uid="{47FF696C-6117-4D2E-A3AB-8820A1E7D9CE}" name="P5" dataDxfId="12"/>
-    <tableColumn id="19" xr3:uid="{FA4923AB-7FF0-492E-A4F0-9612CFE45077}" name="P6" dataDxfId="11"/>
-    <tableColumn id="20" xr3:uid="{25DE5B4A-D987-43FF-A206-BE427E357329}" name="Audio1" dataDxfId="10"/>
-    <tableColumn id="21" xr3:uid="{B4657019-FC58-4700-8EC2-ADEA9DE70938}" name="Audio2" dataDxfId="9"/>
-    <tableColumn id="22" xr3:uid="{ED386123-66EE-47CE-97CB-92713A3243BF}" name="Audio3" dataDxfId="8"/>
-    <tableColumn id="23" xr3:uid="{DEE16AC7-BA35-4A55-BC52-4D717DBC6549}" name="Audio4" dataDxfId="7"/>
-    <tableColumn id="24" xr3:uid="{495ABA16-8114-4F5E-9BC1-18776EEBA69A}" name="Audio5" dataDxfId="6"/>
-    <tableColumn id="25" xr3:uid="{0AB69FD9-D361-475B-A33E-F0EC9EDA4BAE}" name="Audio6" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B71FE2A2-594B-49D5-BF3E-0B87B4A1CCB0}" name="Code" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{99066ED7-FB73-4CE5-BD6D-68B2A16797E7}" name="Langue_fr" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{C5E5BAF6-A992-496A-BC66-B4AF9AA92DD0}" name="Langue_native" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{908B39BA-3596-4F72-8BCF-3C1B2FCCCEF3}" name="Pays" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{1B72A290-5C1E-44A6-A447-200ACF6716B7}" name="Drapeaux" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{C563CC17-226F-4704-AF96-E07E25D95B6B}" name="Sens" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{0725BA7C-155A-4894-A65C-F1E296BE4C5E}" name="Statut1" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{4993FA21-15CF-4114-922A-393B03A69DCE}" name="Statut2" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{14C38812-CC74-499C-952C-386D47399C0E}" name="Statut3" dataDxfId="29"/>
+    <tableColumn id="10" xr3:uid="{877139FF-4465-413E-B07D-E4A10D59F0E3}" name="Statut4" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{F1D42B2E-DB2B-42AF-B635-840FD5759FE4}" name="Statut5" dataDxfId="27"/>
+    <tableColumn id="12" xr3:uid="{14E090AC-24BB-4F19-9BCA-D2ABE2BE0E4F}" name="Statut6" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{AE6452AC-3435-467C-A6C1-280E1815DBC4}" name="Contact" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{3083C17E-EDF2-413A-B542-7CAC44270421}" name="P1" dataDxfId="24"/>
+    <tableColumn id="15" xr3:uid="{326B870C-034B-4A48-A0E2-3B9AA7D7030D}" name="P2" dataDxfId="23"/>
+    <tableColumn id="16" xr3:uid="{25CB2B33-4D8A-449D-8554-52DEFA418EA8}" name="P3" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{90A3021E-E98D-443C-BB21-CF012B0830DB}" name="P4" dataDxfId="21"/>
+    <tableColumn id="18" xr3:uid="{47FF696C-6117-4D2E-A3AB-8820A1E7D9CE}" name="P5" dataDxfId="20"/>
+    <tableColumn id="19" xr3:uid="{FA4923AB-7FF0-492E-A4F0-9612CFE45077}" name="P6" dataDxfId="19"/>
+    <tableColumn id="20" xr3:uid="{25DE5B4A-D987-43FF-A206-BE427E357329}" name="Audio1" dataDxfId="18"/>
+    <tableColumn id="21" xr3:uid="{B4657019-FC58-4700-8EC2-ADEA9DE70938}" name="Audio2" dataDxfId="17"/>
+    <tableColumn id="22" xr3:uid="{ED386123-66EE-47CE-97CB-92713A3243BF}" name="Audio3" dataDxfId="16"/>
+    <tableColumn id="23" xr3:uid="{DEE16AC7-BA35-4A55-BC52-4D717DBC6549}" name="Audio4" dataDxfId="15"/>
+    <tableColumn id="24" xr3:uid="{495ABA16-8114-4F5E-9BC1-18776EEBA69A}" name="Audio5" dataDxfId="14"/>
+    <tableColumn id="25" xr3:uid="{0AB69FD9-D361-475B-A33E-F0EC9EDA4BAE}" name="Audio6" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5606,19 +5634,19 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="M2:X40">
-    <cfRule type="notContainsBlanks" dxfId="33" priority="5">
+  <conditionalFormatting sqref="M2:X42">
+    <cfRule type="notContainsBlanks" dxfId="7" priority="5">
       <formula>LEN(TRIM(M2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:L42">
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"Non traduit"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"Ancienne version"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"Nouvelle version"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Logo Croix-Rouge dans l'en-tête, « PHRASE N » en vert
Le logo officiel remplace le mot « Croix-Rouge » de la ligne de
sous-titre. Comme celui de l'OASIS, il est sur fond blanc et se fond dans
l'en-tête sans détourage. Redimensionné de 1203 à 120 px : 175 Ko pour un
affichage à 28 px n'avaient pas de raison d'être, il en fait 10.

« PHRASE 1 », « PHRASE 2 »… passent au vert de la charte, dans sa version
foncée : tel quel (#9DA679) il n'est qu'à 2,6 de contraste, illisible à
cette taille. La version foncée est à 6,1.

Tiret long remplacé par un tiret simple dans le pied de page.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_traduction.xlsx
+++ b/data_traduction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eulalie.saisset\Documents\1 - Admin\8 - Perso\Oasis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{EB11B65A-6BAD-4DF3-9B39-0FEB10074DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{D5337E19-1860-4516-9A42-2184D86CD86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4545" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1274,7 +1274,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="47">
+  <dxfs count="51">
     <dxf>
       <fill>
         <patternFill>
@@ -1300,6 +1300,34 @@
       <fill>
         <patternFill>
           <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1859,34 +1887,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BBC3B8F8-078D-484B-B353-2EAA17FE9B13}" name="Table1" displayName="Table1" ref="A1:Y42" totalsRowShown="0" headerRowDxfId="45" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BBC3B8F8-078D-484B-B353-2EAA17FE9B13}" name="Table1" displayName="Table1" ref="A1:Y42" totalsRowShown="0" headerRowDxfId="49" dataDxfId="16">
   <autoFilter ref="A1:Y42" xr:uid="{BBC3B8F8-078D-484B-B353-2EAA17FE9B13}"/>
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{B71FE2A2-594B-49D5-BF3E-0B87B4A1CCB0}" name="Code" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{99066ED7-FB73-4CE5-BD6D-68B2A16797E7}" name="Langue_fr" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{C5E5BAF6-A992-496A-BC66-B4AF9AA92DD0}" name="Langue_native" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{908B39BA-3596-4F72-8BCF-3C1B2FCCCEF3}" name="Pays" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{1B72A290-5C1E-44A6-A447-200ACF6716B7}" name="Drapeaux" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{C563CC17-226F-4704-AF96-E07E25D95B6B}" name="Sens" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{0725BA7C-155A-4894-A65C-F1E296BE4C5E}" name="Statut1" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{4993FA21-15CF-4114-922A-393B03A69DCE}" name="Statut2" dataDxfId="30"/>
-    <tableColumn id="9" xr3:uid="{14C38812-CC74-499C-952C-386D47399C0E}" name="Statut3" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{877139FF-4465-413E-B07D-E4A10D59F0E3}" name="Statut4" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{F1D42B2E-DB2B-42AF-B635-840FD5759FE4}" name="Statut5" dataDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{14E090AC-24BB-4F19-9BCA-D2ABE2BE0E4F}" name="Statut6" dataDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{AE6452AC-3435-467C-A6C1-280E1815DBC4}" name="Contact" dataDxfId="25"/>
-    <tableColumn id="14" xr3:uid="{3083C17E-EDF2-413A-B542-7CAC44270421}" name="P1" dataDxfId="24"/>
-    <tableColumn id="15" xr3:uid="{326B870C-034B-4A48-A0E2-3B9AA7D7030D}" name="P2" dataDxfId="23"/>
-    <tableColumn id="16" xr3:uid="{25CB2B33-4D8A-449D-8554-52DEFA418EA8}" name="P3" dataDxfId="22"/>
-    <tableColumn id="17" xr3:uid="{90A3021E-E98D-443C-BB21-CF012B0830DB}" name="P4" dataDxfId="21"/>
-    <tableColumn id="18" xr3:uid="{47FF696C-6117-4D2E-A3AB-8820A1E7D9CE}" name="P5" dataDxfId="20"/>
-    <tableColumn id="19" xr3:uid="{FA4923AB-7FF0-492E-A4F0-9612CFE45077}" name="P6" dataDxfId="19"/>
-    <tableColumn id="20" xr3:uid="{25DE5B4A-D987-43FF-A206-BE427E357329}" name="Audio1" dataDxfId="18"/>
-    <tableColumn id="21" xr3:uid="{B4657019-FC58-4700-8EC2-ADEA9DE70938}" name="Audio2" dataDxfId="17"/>
-    <tableColumn id="22" xr3:uid="{ED386123-66EE-47CE-97CB-92713A3243BF}" name="Audio3" dataDxfId="16"/>
-    <tableColumn id="23" xr3:uid="{DEE16AC7-BA35-4A55-BC52-4D717DBC6549}" name="Audio4" dataDxfId="15"/>
-    <tableColumn id="24" xr3:uid="{495ABA16-8114-4F5E-9BC1-18776EEBA69A}" name="Audio5" dataDxfId="14"/>
-    <tableColumn id="25" xr3:uid="{0AB69FD9-D361-475B-A33E-F0EC9EDA4BAE}" name="Audio6" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{B71FE2A2-594B-49D5-BF3E-0B87B4A1CCB0}" name="Code" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{99066ED7-FB73-4CE5-BD6D-68B2A16797E7}" name="Langue_fr" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{C5E5BAF6-A992-496A-BC66-B4AF9AA92DD0}" name="Langue_native" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{908B39BA-3596-4F72-8BCF-3C1B2FCCCEF3}" name="Pays" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{1B72A290-5C1E-44A6-A447-200ACF6716B7}" name="Drapeaux" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{C563CC17-226F-4704-AF96-E07E25D95B6B}" name="Sens" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{0725BA7C-155A-4894-A65C-F1E296BE4C5E}" name="Statut1" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{4993FA21-15CF-4114-922A-393B03A69DCE}" name="Statut2" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{14C38812-CC74-499C-952C-386D47399C0E}" name="Statut3" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{877139FF-4465-413E-B07D-E4A10D59F0E3}" name="Statut4" dataDxfId="32"/>
+    <tableColumn id="11" xr3:uid="{F1D42B2E-DB2B-42AF-B635-840FD5759FE4}" name="Statut5" dataDxfId="31"/>
+    <tableColumn id="12" xr3:uid="{14E090AC-24BB-4F19-9BCA-D2ABE2BE0E4F}" name="Statut6" dataDxfId="30"/>
+    <tableColumn id="13" xr3:uid="{AE6452AC-3435-467C-A6C1-280E1815DBC4}" name="Contact" dataDxfId="29"/>
+    <tableColumn id="14" xr3:uid="{3083C17E-EDF2-413A-B542-7CAC44270421}" name="P1" dataDxfId="28"/>
+    <tableColumn id="15" xr3:uid="{326B870C-034B-4A48-A0E2-3B9AA7D7030D}" name="P2" dataDxfId="27"/>
+    <tableColumn id="16" xr3:uid="{25CB2B33-4D8A-449D-8554-52DEFA418EA8}" name="P3" dataDxfId="26"/>
+    <tableColumn id="17" xr3:uid="{90A3021E-E98D-443C-BB21-CF012B0830DB}" name="P4" dataDxfId="25"/>
+    <tableColumn id="18" xr3:uid="{47FF696C-6117-4D2E-A3AB-8820A1E7D9CE}" name="P5" dataDxfId="24"/>
+    <tableColumn id="19" xr3:uid="{FA4923AB-7FF0-492E-A4F0-9612CFE45077}" name="P6" dataDxfId="23"/>
+    <tableColumn id="20" xr3:uid="{25DE5B4A-D987-43FF-A206-BE427E357329}" name="Audio1" dataDxfId="22"/>
+    <tableColumn id="21" xr3:uid="{B4657019-FC58-4700-8EC2-ADEA9DE70938}" name="Audio2" dataDxfId="21"/>
+    <tableColumn id="22" xr3:uid="{ED386123-66EE-47CE-97CB-92713A3243BF}" name="Audio3" dataDxfId="20"/>
+    <tableColumn id="23" xr3:uid="{DEE16AC7-BA35-4A55-BC52-4D717DBC6549}" name="Audio4" dataDxfId="19"/>
+    <tableColumn id="24" xr3:uid="{495ABA16-8114-4F5E-9BC1-18776EEBA69A}" name="Audio5" dataDxfId="18"/>
+    <tableColumn id="25" xr3:uid="{0AB69FD9-D361-475B-A33E-F0EC9EDA4BAE}" name="Audio6" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5635,18 +5663,18 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="M2:X42">
-    <cfRule type="notContainsBlanks" dxfId="7" priority="5">
-      <formula>LEN(TRIM(M2))&gt;0</formula>
+    <cfRule type="containsBlanks" dxfId="4" priority="6">
+      <formula>LEN(TRIM(M2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:L42">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"Non traduit"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>"Ancienne version"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Nouvelle version"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Enregistrements en farsi, importés du Drive
Sur les 30 fichiers de l'archive, 25 sont rigoureusement identiques à ceux
déjà présents (comparaison par empreinte, pas par date) : arabe, arménien,
pachto, peul et russe étaient déjà à jour. Le farsi est le seul apport,
5 phrases.

Quatre des cinq fichiers farsi n'avaient pas d'extension ; leur en-tête
binaire les donne en m4a, ils sont renommés en conséquence.

Le farsi n'a aucune traduction écrite : la personne verra « Traduction à
ajouter » mais pourra écouter les 5 phrases, ce que le site prévoit.

Archives d'import exclues du dépôt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_traduction.xlsx
+++ b/data_traduction.xlsx
@@ -2772,11 +2772,31 @@
       <c r="Q14" s="13" t="n"/>
       <c r="R14" s="13" t="n"/>
       <c r="S14" s="13" t="n"/>
-      <c r="T14" s="13" t="n"/>
-      <c r="U14" s="13" t="n"/>
-      <c r="V14" s="13" t="n"/>
-      <c r="W14" s="13" t="n"/>
-      <c r="X14" s="13" t="n"/>
+      <c r="T14" s="13" t="inlineStr">
+        <is>
+          <t>audio/fa_p1.m4a</t>
+        </is>
+      </c>
+      <c r="U14" s="13" t="inlineStr">
+        <is>
+          <t>audio/fa_p2.m4a</t>
+        </is>
+      </c>
+      <c r="V14" s="13" t="inlineStr">
+        <is>
+          <t>audio/fa_p3.m4a</t>
+        </is>
+      </c>
+      <c r="W14" s="13" t="inlineStr">
+        <is>
+          <t>audio/fa_p4.m4a</t>
+        </is>
+      </c>
+      <c r="X14" s="13" t="inlineStr">
+        <is>
+          <t>audio/fa_p5.m4a</t>
+        </is>
+      </c>
       <c r="Y14" s="13" t="n"/>
     </row>
     <row r="15">

</xml_diff>